<commit_message>
add extrusion and stiffener takeoffs
</commit_message>
<xml_diff>
--- a/01_storefront_acm_elevation_set.xlsx
+++ b/01_storefront_acm_elevation_set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\brand\source\AgentRepos\PanelNester\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230C889A-079C-4AF5-8004-0F752CBD7C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C2AEE3-3367-42D9-8ECC-8B0F1B3AD86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36920" yWindow="1510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36960" yWindow="1470" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ImportData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="18">
   <si>
     <t>Id</t>
   </si>
@@ -80,7 +80,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,6 +100,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -164,8 +170,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ImportTable" displayName="ImportTable" ref="A1:F9">
-  <autoFilter ref="A1:F9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ImportTable" displayName="ImportTable" ref="A1:F12">
+  <autoFilter ref="A1:F12" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Length"/>
@@ -463,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -651,7 +657,68 @@
         <v>16</v>
       </c>
     </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="2">
+        <v>24</v>
+      </c>
+      <c r="C10" s="2">
+        <v>96</v>
+      </c>
+      <c r="D10" s="3">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2">
+        <v>18</v>
+      </c>
+      <c r="C11" s="2">
+        <v>42</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="2">
+        <v>30</v>
+      </c>
+      <c r="C12" s="2">
+        <v>96</v>
+      </c>
+      <c r="D12" s="3">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>